<commit_message>
ALTS_Excel_INVOICE1.xslx and ALTS_TUTORIAL1.xlsx current versions replace
The uploaded files replace the stale versions. This is because the files were updated to create versions 2 and 3. ALTS_Excel_INVOICE1.xslx and ALTS_TUTORIAL1.xlsx
</commit_message>
<xml_diff>
--- a/ALTS_Excel_INVOICE1.xlsx
+++ b/ALTS_Excel_INVOICE1.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30327"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30408"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3FA4EEB8-431C-452B-8F40-CE4EBABA6328}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{92F0578F-B9E3-498A-BC08-C329ED9FF270}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,8 +31,49 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>tc={74B194F1-706C-4D16-B8CF-841F3FE0ACD5}</author>
+  </authors>
+  <commentList>
+    <comment ref="D21" authorId="0" shapeId="0" xr:uid="{74B194F1-706C-4D16-B8CF-841F3FE0ACD5}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    This formula can also be used here:
+=IF(SUM(InvoiceTable[AMOUNT])=0, "", SUM(InvoiceTable[AMOUNT]))</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="32">
   <si>
     <t>INVOICE</t>
   </si>
@@ -61,34 +102,34 @@
     <t>Row_ID</t>
   </si>
   <si>
-    <t>ICTS</t>
-  </si>
-  <si>
-    <t>ITS_2026_1030</t>
-  </si>
-  <si>
-    <t>Khusa Marketing</t>
-  </si>
-  <si>
-    <t>123 Aba Owerri Road</t>
-  </si>
-  <si>
-    <t>CUSTOMER ID</t>
-  </si>
-  <si>
-    <t>TERMS</t>
+    <t>AddressLine1</t>
+  </si>
+  <si>
+    <t>AddressLine2</t>
+  </si>
+  <si>
+    <t>AddressLine3</t>
+  </si>
+  <si>
+    <t>FDL</t>
+  </si>
+  <si>
+    <t>ITS_2026_1050</t>
+  </si>
+  <si>
+    <t>12 Ugbana Lane</t>
   </si>
   <si>
     <t>Aba, Abia State</t>
   </si>
   <si>
-    <t>Due upon receipt</t>
-  </si>
-  <si>
-    <t>+234 804 678 4565</t>
-  </si>
-  <si>
-    <t>ijegho@ictsl.com</t>
+    <t>COMPANY ACCOUNT DETAILS</t>
+  </si>
+  <si>
+    <t>ICT SOLUTIONS LIMITED</t>
+  </si>
+  <si>
+    <t>Arondizuogu Community Bank =&gt; 20337886565</t>
   </si>
   <si>
     <t>DESCRIPTION</t>
@@ -103,22 +144,10 @@
     <t>AMOUNT</t>
   </si>
   <si>
-    <t>c</t>
-  </si>
-  <si>
-    <t>Helmets</t>
-  </si>
-  <si>
-    <t>Labor: 5 hours at 1800/hr</t>
-  </si>
-  <si>
-    <t>New client discount</t>
-  </si>
-  <si>
-    <t>Dotted Hand Gloves</t>
-  </si>
-  <si>
-    <t>Safety Boots</t>
+    <t>M365 Subscription</t>
+  </si>
+  <si>
+    <t>Internet Service Subscription</t>
   </si>
   <si>
     <t>Thanks for partnering with us.</t>
@@ -150,7 +179,7 @@
     <numFmt numFmtId="164" formatCode="[$₦-470]#,##0.00;\-[$₦-470]#,##0.00"/>
     <numFmt numFmtId="165" formatCode="[$-409]d\-mmm\-yyyy;@"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="16">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -234,6 +263,29 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF242424"/>
+      <name val="Aptos Narrow"/>
+      <charset val="1"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -255,7 +307,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -343,12 +395,21 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment readingOrder="1"/>
@@ -356,22 +417,13 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" readingOrder="1"/>
-    </xf>
     <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment readingOrder="1"/>
     </xf>
     <xf numFmtId="10" fontId="5" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment readingOrder="1"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment readingOrder="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment readingOrder="1"/>
     </xf>
     <xf numFmtId="164" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
@@ -422,16 +474,24 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment readingOrder="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment readingOrder="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="3" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment readingOrder="1"/>
     </xf>
@@ -449,6 +509,9 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" readingOrder="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -466,6 +529,11 @@
           <bgColor rgb="FFF5F5F5"/>
         </patternFill>
       </fill>
+      <border>
+        <right style="thin">
+          <color rgb="FF000000"/>
+        </right>
+      </border>
     </dxf>
     <dxf>
       <font>
@@ -529,7 +597,7 @@
         <shadow val="0"/>
         <u val="none"/>
         <vertAlign val="baseline"/>
-        <sz val="10"/>
+        <sz val="11"/>
         <color theme="1"/>
         <name val="Arial"/>
         <charset val="1"/>
@@ -794,9 +862,15 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <person displayName="Leonard Mbibi" id="{32788DE4-B660-4693-AC8A-21FDCCBD6781}" userId="S::leonard.mbibi@gregobyte.com::02c0729d-909c-4f02-970f-b0082d86fea3" providerId="AD"/>
+</personList>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{CB748B29-1419-4A8B-82C8-2906DFB1F144}" name="InvoiceTable" displayName="InvoiceTable" ref="A15:E21" totalsRowShown="0" headerRowDxfId="14" headerRowBorderDxfId="12" tableBorderDxfId="13" totalsRowBorderDxfId="11">
-  <autoFilter ref="A15:E21" xr:uid="{CB748B29-1419-4A8B-82C8-2906DFB1F144}">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{CB748B29-1419-4A8B-82C8-2906DFB1F144}" name="InvoiceTable" displayName="InvoiceTable" ref="A14:E20" totalsRowShown="0" headerRowDxfId="14" headerRowBorderDxfId="12" tableBorderDxfId="13" totalsRowBorderDxfId="11">
+  <autoFilter ref="A14:E20" xr:uid="{CB748B29-1419-4A8B-82C8-2906DFB1F144}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
@@ -810,22 +884,27 @@
     <tableColumn id="5" xr3:uid="{5E1B32BD-13E3-4DFA-AF31-2B1EA87F074E}" name="AMOUNT" dataDxfId="9">
       <calculatedColumnFormula>IF(OR(InvoiceTable[[#This Row],[UNIT PRICE]]="", InvoiceTable[[#This Row],[DESCRIPTION]]=""), "", IF(InvoiceTable[[#This Row],[QTY]]="", InvoiceTable[[#This Row],[UNIT PRICE]], InvoiceTable[[#This Row],[QTY]]*InvoiceTable[[#This Row],[UNIT PRICE]]))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{C3592BDE-6C53-451A-9DDD-C87FF4C5589F}" name="c" dataDxfId="8"/>
+    <tableColumn id="2" xr3:uid="{C3592BDE-6C53-451A-9DDD-C87FF4C5589F}" name="Row_ID" dataDxfId="8">
+      <calculatedColumnFormula>ROW() - ROW(InvoiceTable[[#Headers],[Row_ID]])</calculatedColumnFormula>
+    </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{EEC8D22E-B88A-42FA-BCA6-0ADB538DF19F}" name="InvoiceNumberTable" displayName="InvoiceNumberTable" ref="A7:E8" totalsRowShown="0" headerRowBorderDxfId="6" tableBorderDxfId="7" totalsRowBorderDxfId="5">
-  <autoFilter ref="A7:E8" xr:uid="{EEC8D22E-B88A-42FA-BCA6-0ADB538DF19F}">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{EEC8D22E-B88A-42FA-BCA6-0ADB538DF19F}" name="InvoiceNumberTable" displayName="InvoiceNumberTable" ref="A7:H8" totalsRowShown="0" headerRowBorderDxfId="6" tableBorderDxfId="7" totalsRowBorderDxfId="5">
+  <autoFilter ref="A7:H8" xr:uid="{EEC8D22E-B88A-42FA-BCA6-0ADB538DF19F}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
     <filterColumn colId="3" hiddenButton="1"/>
     <filterColumn colId="4" hiddenButton="1"/>
+    <filterColumn colId="5" hiddenButton="1"/>
+    <filterColumn colId="6" hiddenButton="1"/>
+    <filterColumn colId="7" hiddenButton="1"/>
   </autoFilter>
-  <tableColumns count="5">
+  <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{44E30872-04A8-4BF4-9D71-76FEC2FAAB2E}" name="BILL_T0" dataDxfId="4"/>
     <tableColumn id="2" xr3:uid="{4977195D-75B6-4433-A4A8-1F9A9F32B3D2}" name="Bill_No" dataDxfId="3"/>
     <tableColumn id="3" xr3:uid="{7845B608-7FC8-4FE3-BB5D-9E412DBBF56B}" name="INVOICE_No" dataDxfId="2"/>
@@ -833,6 +912,9 @@
       <calculatedColumnFormula>TODAY()</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="5" xr3:uid="{F847AC23-4D8D-4B7A-AE33-5F496312EAA1}" name="Row_ID" dataDxfId="0"/>
+    <tableColumn id="6" xr3:uid="{27F3F0F8-987B-4B04-B7E7-6263087FC14B}" name="AddressLine1"/>
+    <tableColumn id="7" xr3:uid="{5579A75A-422C-449B-8425-61A1BAA57925}" name="AddressLine2"/>
+    <tableColumn id="8" xr3:uid="{2AAC3AFA-7A23-4B60-9DF2-DCF9ADF5A78F}" name="AddressLine3"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
 </table>
@@ -1133,63 +1215,73 @@
 </a:theme>
 </file>
 
+<file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
+<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="D21" dT="2026-08-12T14:00:18.67" personId="{32788DE4-B660-4693-AC8A-21FDCCBD6781}" id="{74B194F1-706C-4D16-B8CF-841F3FE0ACD5}">
+    <text>This formula can also be used here:
+=IF(SUM(InvoiceTable[AMOUNT])=0, "", SUM(InvoiceTable[AMOUNT]))</text>
+  </threadedComment>
+</ThreadedComments>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A2:E30"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A2:H29"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="31.42578125" customWidth="1"/>
-    <col min="2" max="2" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="28.28515625" customWidth="1"/>
+    <col min="2" max="2" width="9" customWidth="1"/>
     <col min="3" max="3" width="14.140625" customWidth="1"/>
-    <col min="4" max="4" width="23.42578125" customWidth="1"/>
+    <col min="4" max="4" width="27" customWidth="1"/>
     <col min="5" max="5" width="7.140625" customWidth="1"/>
+    <col min="6" max="8" width="0" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:5" ht="48" customHeight="1">
-      <c r="A2" s="27"/>
-      <c r="B2" s="12"/>
-      <c r="C2" s="36" t="s">
+    <row r="2" spans="1:8" ht="48" customHeight="1">
+      <c r="A2" s="24"/>
+      <c r="B2" s="9"/>
+      <c r="C2" s="37" t="s">
         <v>0</v>
       </c>
-      <c r="D2" s="36"/>
-      <c r="E2" s="24"/>
-    </row>
-    <row r="3" spans="1:5">
-      <c r="A3" s="13" t="s">
+      <c r="D2" s="37"/>
+      <c r="E2" s="21"/>
+    </row>
+    <row r="3" spans="1:8">
+      <c r="A3" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="35"/>
-      <c r="C3" s="35"/>
+      <c r="B3" s="36"/>
+      <c r="C3" s="36"/>
       <c r="D3" s="1"/>
-      <c r="E3" s="21"/>
-    </row>
-    <row r="4" spans="1:5">
-      <c r="A4" s="13" t="s">
+      <c r="E3" s="18"/>
+    </row>
+    <row r="4" spans="1:8">
+      <c r="A4" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="35"/>
-      <c r="C4" s="35"/>
+      <c r="B4" s="36"/>
+      <c r="C4" s="36"/>
       <c r="D4" s="1"/>
-      <c r="E4" s="21"/>
-    </row>
-    <row r="5" spans="1:5">
-      <c r="A5" s="13" t="s">
+      <c r="E4" s="18"/>
+    </row>
+    <row r="5" spans="1:8">
+      <c r="A5" s="10" t="s">
         <v>3</v>
       </c>
       <c r="B5" s="1"/>
       <c r="C5" s="1"/>
       <c r="D5" s="1"/>
-      <c r="E5" s="21"/>
-    </row>
-    <row r="6" spans="1:5">
-      <c r="A6" s="14"/>
+      <c r="E5" s="18"/>
+    </row>
+    <row r="6" spans="1:8">
+      <c r="A6" s="11"/>
       <c r="B6" s="1"/>
       <c r="C6" s="1"/>
-      <c r="D6" s="1"/>
-      <c r="E6" s="21"/>
-    </row>
-    <row r="7" spans="1:5">
-      <c r="A7" s="15" t="s">
+      <c r="D6" s="29"/>
+      <c r="E6" s="18"/>
+    </row>
+    <row r="7" spans="1:8">
+      <c r="A7" s="12" t="s">
         <v>4</v>
       </c>
       <c r="B7" s="2" t="s">
@@ -1201,302 +1293,301 @@
       <c r="D7" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E7" s="25" t="s">
+      <c r="E7" s="22" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="8" spans="1:5">
-      <c r="A8" s="28" t="s">
+      <c r="F7" s="30" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="29">
-        <v>1030</v>
-      </c>
-      <c r="C8" s="30" t="s">
+      <c r="G7" s="31" t="s">
         <v>10</v>
       </c>
-      <c r="D8" s="31">
+      <c r="H7" s="30" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8">
+      <c r="A8" s="25" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8" s="28">
+        <v>1050</v>
+      </c>
+      <c r="C8" s="26" t="s">
+        <v>13</v>
+      </c>
+      <c r="D8" s="27">
         <f ca="1">TODAY()</f>
-        <v>46241</v>
-      </c>
-      <c r="E8" s="32">
+        <v>46249</v>
+      </c>
+      <c r="E8" s="33">
         <v>1</v>
       </c>
-    </row>
-    <row r="9" spans="1:5">
-      <c r="A9" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="B9" s="35"/>
-      <c r="C9" s="35"/>
+      <c r="F8" t="s">
+        <v>14</v>
+      </c>
+      <c r="G8" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8">
+      <c r="A9" s="13" t="str" cm="1">
+        <f t="array" ref="A9">IF(InvoiceNumberTable[AddressLine1] = "", "", InvoiceNumberTable[AddressLine1])</f>
+        <v>12 Ugbana Lane</v>
+      </c>
+      <c r="B9" s="36"/>
+      <c r="C9" s="36"/>
       <c r="D9" s="1"/>
-      <c r="E9" s="21"/>
-    </row>
-    <row r="10" spans="1:5">
-      <c r="A10" s="16" t="s">
-        <v>12</v>
+      <c r="E9" s="18"/>
+    </row>
+    <row r="10" spans="1:8">
+      <c r="A10" s="13" t="str" cm="1">
+        <f t="array" ref="A10">IF(InvoiceNumberTable[AddressLine2] = "", "", InvoiceNumberTable[AddressLine2])</f>
+        <v>Aba, Abia State</v>
       </c>
       <c r="B10" s="1"/>
-      <c r="C10" s="2" t="s">
-        <v>13</v>
-      </c>
+      <c r="C10" s="2"/>
       <c r="D10" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E10" s="26"/>
-    </row>
-    <row r="11" spans="1:5">
-      <c r="A11" s="16" t="s">
-        <v>15</v>
+        <v>16</v>
+      </c>
+      <c r="E10" s="23"/>
+    </row>
+    <row r="11" spans="1:8">
+      <c r="A11" s="13" t="str" cm="1">
+        <f t="array" ref="A11">IF(InvoiceNumberTable[AddressLine3] = "", "", InvoiceNumberTable[AddressLine3])</f>
+        <v/>
       </c>
       <c r="B11" s="1"/>
-      <c r="C11" s="8">
-        <v>100</v>
-      </c>
-      <c r="D11" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="E11" s="21"/>
-    </row>
-    <row r="12" spans="1:5">
-      <c r="A12" s="16" t="s">
+      <c r="C11" s="40" t="s">
         <v>17</v>
       </c>
-      <c r="B12" s="35"/>
-      <c r="C12" s="35"/>
-      <c r="D12" s="1"/>
-      <c r="E12" s="21"/>
-    </row>
-    <row r="13" spans="1:5">
-      <c r="A13" s="17" t="s">
+      <c r="D11" s="40"/>
+      <c r="E11" s="18"/>
+    </row>
+    <row r="12" spans="1:8">
+      <c r="A12" s="14"/>
+      <c r="B12" s="1"/>
+      <c r="C12" s="40" t="s">
         <v>18</v>
       </c>
-      <c r="B13" s="35"/>
-      <c r="C13" s="35"/>
+      <c r="D12" s="40"/>
+      <c r="E12" s="18"/>
+    </row>
+    <row r="13" spans="1:8">
+      <c r="A13" s="11"/>
+      <c r="B13" s="36"/>
+      <c r="C13" s="36"/>
       <c r="D13" s="1"/>
-      <c r="E13" s="21"/>
-    </row>
-    <row r="14" spans="1:5">
-      <c r="A14" s="14"/>
-      <c r="B14" s="35"/>
-      <c r="C14" s="35"/>
-      <c r="D14" s="1"/>
-      <c r="E14" s="21"/>
-    </row>
-    <row r="15" spans="1:5">
-      <c r="A15" s="15" t="s">
+      <c r="E13" s="18"/>
+    </row>
+    <row r="14" spans="1:8">
+      <c r="A14" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="B14" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="C15" s="2" t="s">
+      <c r="C14" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="D15" s="2" t="s">
+      <c r="D14" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="E15" s="25" t="s">
+      <c r="E14" s="22" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8">
+      <c r="A15" s="13" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="16" spans="1:5">
-      <c r="A16" s="16" t="s">
+      <c r="B15" s="5">
+        <v>2</v>
+      </c>
+      <c r="C15" s="3">
+        <v>1700378</v>
+      </c>
+      <c r="D15" s="3">
+        <f>IF(OR(InvoiceTable[[#This Row],[UNIT PRICE]]="", InvoiceTable[[#This Row],[DESCRIPTION]]=""), "", IF(InvoiceTable[[#This Row],[QTY]]="", InvoiceTable[[#This Row],[UNIT PRICE]], InvoiceTable[[#This Row],[QTY]]*InvoiceTable[[#This Row],[UNIT PRICE]]))</f>
+        <v>3400756</v>
+      </c>
+      <c r="E15" s="20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8">
+      <c r="A16" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="B16" s="7">
-        <v>120</v>
-      </c>
-      <c r="C16" s="4">
-        <v>4500</v>
-      </c>
-      <c r="D16" s="4">
+      <c r="B16" s="5">
+        <v>3</v>
+      </c>
+      <c r="C16" s="3">
+        <v>50000</v>
+      </c>
+      <c r="D16" s="3">
         <f>IF(OR(InvoiceTable[[#This Row],[UNIT PRICE]]="", InvoiceTable[[#This Row],[DESCRIPTION]]=""), "", IF(InvoiceTable[[#This Row],[QTY]]="", InvoiceTable[[#This Row],[UNIT PRICE]], InvoiceTable[[#This Row],[QTY]]*InvoiceTable[[#This Row],[UNIT PRICE]]))</f>
-        <v>540000</v>
-      </c>
-      <c r="E16" s="23"/>
+        <v>150000</v>
+      </c>
+      <c r="E16" s="20">
+        <v>2</v>
+      </c>
     </row>
     <row r="17" spans="1:5">
-      <c r="A17" s="16" t="s">
-        <v>25</v>
-      </c>
-      <c r="B17" s="7">
-        <v>5</v>
-      </c>
-      <c r="C17" s="4">
-        <v>75</v>
-      </c>
-      <c r="D17" s="4">
-        <f>IF(OR(InvoiceTable[[#This Row],[UNIT PRICE]]="", InvoiceTable[[#This Row],[DESCRIPTION]]=""), "", IF(InvoiceTable[[#This Row],[QTY]]="", InvoiceTable[[#This Row],[UNIT PRICE]], InvoiceTable[[#This Row],[QTY]]*InvoiceTable[[#This Row],[UNIT PRICE]]))</f>
-        <v>375</v>
-      </c>
-      <c r="E17" s="23"/>
-    </row>
-    <row r="18" spans="1:5">
-      <c r="A18" s="16" t="s">
-        <v>26</v>
-      </c>
-      <c r="B18" s="1"/>
-      <c r="C18" s="4">
-        <v>-50</v>
-      </c>
-      <c r="D18" s="4">
-        <f>IF(OR(InvoiceTable[[#This Row],[UNIT PRICE]]="", InvoiceTable[[#This Row],[DESCRIPTION]]=""), "", IF(InvoiceTable[[#This Row],[QTY]]="", InvoiceTable[[#This Row],[UNIT PRICE]], InvoiceTable[[#This Row],[QTY]]*InvoiceTable[[#This Row],[UNIT PRICE]]))</f>
-        <v>-50</v>
-      </c>
-      <c r="E18" s="23"/>
-    </row>
-    <row r="19" spans="1:5">
-      <c r="A19" s="14" t="s">
-        <v>27</v>
-      </c>
-      <c r="B19" s="1">
-        <v>3</v>
-      </c>
-      <c r="C19" s="4">
-        <v>10000</v>
-      </c>
-      <c r="D19" s="4">
-        <f>IF(OR(InvoiceTable[[#This Row],[UNIT PRICE]]="", InvoiceTable[[#This Row],[DESCRIPTION]]=""), "", IF(InvoiceTable[[#This Row],[QTY]]="", InvoiceTable[[#This Row],[UNIT PRICE]], InvoiceTable[[#This Row],[QTY]]*InvoiceTable[[#This Row],[UNIT PRICE]]))</f>
-        <v>30000</v>
-      </c>
-      <c r="E19" s="23"/>
-    </row>
-    <row r="20" spans="1:5">
-      <c r="A20" s="14" t="s">
-        <v>28</v>
-      </c>
-      <c r="B20" s="1">
-        <v>150</v>
-      </c>
-      <c r="C20" s="9">
-        <v>12000</v>
-      </c>
-      <c r="D20" s="4">
-        <f>IF(OR(InvoiceTable[[#This Row],[UNIT PRICE]]="", InvoiceTable[[#This Row],[DESCRIPTION]]=""), "", IF(InvoiceTable[[#This Row],[QTY]]="", InvoiceTable[[#This Row],[UNIT PRICE]], InvoiceTable[[#This Row],[QTY]]*InvoiceTable[[#This Row],[UNIT PRICE]]))</f>
-        <v>1800000</v>
-      </c>
-      <c r="E20" s="23"/>
-    </row>
-    <row r="21" spans="1:5">
-      <c r="A21" s="14"/>
-      <c r="B21" s="1"/>
-      <c r="C21" s="9"/>
-      <c r="D21" s="4" t="str">
+      <c r="A17" s="13"/>
+      <c r="B17" s="1"/>
+      <c r="C17" s="3"/>
+      <c r="D17" s="3" t="str">
         <f>IF(OR(InvoiceTable[[#This Row],[UNIT PRICE]]="", InvoiceTable[[#This Row],[DESCRIPTION]]=""), "", IF(InvoiceTable[[#This Row],[QTY]]="", InvoiceTable[[#This Row],[UNIT PRICE]], InvoiceTable[[#This Row],[QTY]]*InvoiceTable[[#This Row],[UNIT PRICE]]))</f>
         <v/>
       </c>
-      <c r="E21" s="23"/>
+      <c r="E17" s="20">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5">
+      <c r="A18" s="11"/>
+      <c r="B18" s="1"/>
+      <c r="C18" s="3"/>
+      <c r="D18" s="3" t="str">
+        <f>IF(OR(InvoiceTable[[#This Row],[UNIT PRICE]]="", InvoiceTable[[#This Row],[DESCRIPTION]]=""), "", IF(InvoiceTable[[#This Row],[QTY]]="", InvoiceTable[[#This Row],[UNIT PRICE]], InvoiceTable[[#This Row],[QTY]]*InvoiceTable[[#This Row],[UNIT PRICE]]))</f>
+        <v/>
+      </c>
+      <c r="E18" s="20">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5">
+      <c r="A19" s="11"/>
+      <c r="B19" s="1"/>
+      <c r="C19" s="6"/>
+      <c r="D19" s="3" t="str">
+        <f>IF(OR(InvoiceTable[[#This Row],[UNIT PRICE]]="", InvoiceTable[[#This Row],[DESCRIPTION]]=""), "", IF(InvoiceTable[[#This Row],[QTY]]="", InvoiceTable[[#This Row],[UNIT PRICE]], InvoiceTable[[#This Row],[QTY]]*InvoiceTable[[#This Row],[UNIT PRICE]]))</f>
+        <v/>
+      </c>
+      <c r="E19" s="20">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5">
+      <c r="A20" s="11"/>
+      <c r="B20" s="1"/>
+      <c r="C20" s="6"/>
+      <c r="D20" s="3" t="str">
+        <f>IF(OR(InvoiceTable[[#This Row],[UNIT PRICE]]="", InvoiceTable[[#This Row],[DESCRIPTION]]=""), "", IF(InvoiceTable[[#This Row],[QTY]]="", InvoiceTable[[#This Row],[UNIT PRICE]], InvoiceTable[[#This Row],[QTY]]*InvoiceTable[[#This Row],[UNIT PRICE]]))</f>
+        <v/>
+      </c>
+      <c r="E20" s="20">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5">
+      <c r="A21" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="B21" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="C21" s="5"/>
+      <c r="D21" s="3">
+        <f>IF(INDEX(InvoiceTable[AMOUNT], 1)="", "", SUM(InvoiceTable[AMOUNT]))</f>
+        <v>3550756</v>
+      </c>
+      <c r="E21" s="18"/>
     </row>
     <row r="22" spans="1:5">
-      <c r="A22" s="18" t="s">
+      <c r="A22" s="11"/>
+      <c r="B22" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C22" s="5"/>
+      <c r="D22" s="4">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="E22" s="18"/>
+    </row>
+    <row r="23" spans="1:5">
+      <c r="A23" s="11"/>
+      <c r="B23" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="C23" s="5"/>
+      <c r="D23" s="3">
+        <f>IF(D21="", "", D21 * D22)</f>
+        <v>248552.92</v>
+      </c>
+      <c r="E23" s="18"/>
+    </row>
+    <row r="24" spans="1:5" ht="24">
+      <c r="A24" s="11"/>
+      <c r="B24" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="B22" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="C22" s="7"/>
-      <c r="D22" s="4">
-        <f>SUM(D16:D21)</f>
-        <v>2370325</v>
-      </c>
-      <c r="E22" s="21"/>
-    </row>
-    <row r="23" spans="1:5">
-      <c r="A23" s="14"/>
-      <c r="B23" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="C23" s="7"/>
-      <c r="D23" s="5">
-        <v>7.0000000000000007E-2</v>
-      </c>
-      <c r="E23" s="21"/>
-    </row>
-    <row r="24" spans="1:5">
-      <c r="A24" s="14"/>
-      <c r="B24" s="7" t="s">
-        <v>32</v>
-      </c>
       <c r="C24" s="7"/>
-      <c r="D24" s="4">
-        <f>D23*D22</f>
-        <v>165922.75000000003</v>
-      </c>
-      <c r="E24" s="21"/>
-    </row>
-    <row r="25" spans="1:5" ht="24">
-      <c r="A25" s="14"/>
-      <c r="B25" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="C25" s="10"/>
-      <c r="D25" s="6">
-        <f>D22+D24</f>
-        <v>2536247.75</v>
-      </c>
-      <c r="E25" s="11"/>
+      <c r="D24" s="32">
+        <f>IF(D21 = "", "", D21+D23)</f>
+        <v>3799308.92</v>
+      </c>
+      <c r="E24" s="8"/>
+    </row>
+    <row r="25" spans="1:5">
+      <c r="A25" s="11"/>
+      <c r="B25" s="1"/>
+      <c r="C25" s="1"/>
+      <c r="D25" s="1"/>
+      <c r="E25" s="18"/>
     </row>
     <row r="26" spans="1:5">
-      <c r="A26" s="14"/>
+      <c r="A26" s="11"/>
       <c r="B26" s="1"/>
       <c r="C26" s="1"/>
       <c r="D26" s="1"/>
-      <c r="E26" s="21"/>
+      <c r="E26" s="18"/>
     </row>
     <row r="27" spans="1:5">
-      <c r="A27" s="14"/>
-      <c r="B27" s="1"/>
-      <c r="C27" s="1"/>
-      <c r="D27" s="1"/>
-      <c r="E27" s="21"/>
+      <c r="A27" s="38" t="s">
+        <v>30</v>
+      </c>
+      <c r="B27" s="39"/>
+      <c r="C27" s="39"/>
+      <c r="D27" s="39"/>
+      <c r="E27" s="18"/>
     </row>
     <row r="28" spans="1:5">
-      <c r="A28" s="37" t="s">
-        <v>34</v>
-      </c>
-      <c r="B28" s="38"/>
-      <c r="C28" s="38"/>
-      <c r="D28" s="38"/>
-      <c r="E28" s="21"/>
+      <c r="A28" s="34" t="s">
+        <v>31</v>
+      </c>
+      <c r="B28" s="35"/>
+      <c r="C28" s="35"/>
+      <c r="D28" s="35"/>
+      <c r="E28" s="18"/>
     </row>
     <row r="29" spans="1:5">
-      <c r="A29" s="33" t="s">
-        <v>35</v>
-      </c>
-      <c r="B29" s="34"/>
-      <c r="C29" s="34"/>
-      <c r="D29" s="34"/>
-      <c r="E29" s="21"/>
-    </row>
-    <row r="30" spans="1:5">
-      <c r="A30" s="19"/>
-      <c r="B30" s="20"/>
-      <c r="C30" s="20"/>
-      <c r="D30" s="20"/>
-      <c r="E30" s="22"/>
+      <c r="A29" s="16"/>
+      <c r="B29" s="17"/>
+      <c r="C29" s="17"/>
+      <c r="D29" s="17"/>
+      <c r="E29" s="19"/>
     </row>
   </sheetData>
   <sheetProtection formatCells="0" insertRows="0" autoFilter="0"/>
   <protectedRanges>
-    <protectedRange sqref="A16:C21" name="UserInput"/>
+    <protectedRange sqref="A15:C20" name="UserInput"/>
   </protectedRanges>
   <mergeCells count="9">
-    <mergeCell ref="A29:D29"/>
+    <mergeCell ref="A28:D28"/>
     <mergeCell ref="B13:C13"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="B12:C12"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B3:C3"/>
     <mergeCell ref="B4:C4"/>
     <mergeCell ref="B9:C9"/>
-    <mergeCell ref="A28:D28"/>
+    <mergeCell ref="A27:D27"/>
+    <mergeCell ref="C11:D11"/>
+    <mergeCell ref="C12:D12"/>
   </mergeCells>
-  <hyperlinks>
-    <hyperlink ref="A13" r:id="rId1" xr:uid="{4467A923-BBDD-4696-987C-7316B9841A21}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId2"/>
+  <drawing r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
   <tableParts count="2">
     <tablePart r:id="rId3"/>
     <tablePart r:id="rId4"/>

</xml_diff>

<commit_message>
ALTS_Excel_INVOICE1.xslx and ALTS_TUTORIAL1.xlsx overwritten
ALTS_Excel_INVOICE1.xslx and ALTS_TUTORIAL1.xlsx had changes to achieve versions 2 and 3.
</commit_message>
<xml_diff>
--- a/ALTS_Excel_INVOICE1.xlsx
+++ b/ALTS_Excel_INVOICE1.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30327"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30408"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3FA4EEB8-431C-452B-8F40-CE4EBABA6328}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{92F0578F-B9E3-498A-BC08-C329ED9FF270}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,8 +31,49 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>tc={74B194F1-706C-4D16-B8CF-841F3FE0ACD5}</author>
+  </authors>
+  <commentList>
+    <comment ref="D21" authorId="0" shapeId="0" xr:uid="{74B194F1-706C-4D16-B8CF-841F3FE0ACD5}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    This formula can also be used here:
+=IF(SUM(InvoiceTable[AMOUNT])=0, "", SUM(InvoiceTable[AMOUNT]))</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="32">
   <si>
     <t>INVOICE</t>
   </si>
@@ -61,34 +102,34 @@
     <t>Row_ID</t>
   </si>
   <si>
-    <t>ICTS</t>
-  </si>
-  <si>
-    <t>ITS_2026_1030</t>
-  </si>
-  <si>
-    <t>Khusa Marketing</t>
-  </si>
-  <si>
-    <t>123 Aba Owerri Road</t>
-  </si>
-  <si>
-    <t>CUSTOMER ID</t>
-  </si>
-  <si>
-    <t>TERMS</t>
+    <t>AddressLine1</t>
+  </si>
+  <si>
+    <t>AddressLine2</t>
+  </si>
+  <si>
+    <t>AddressLine3</t>
+  </si>
+  <si>
+    <t>FDL</t>
+  </si>
+  <si>
+    <t>ITS_2026_1050</t>
+  </si>
+  <si>
+    <t>12 Ugbana Lane</t>
   </si>
   <si>
     <t>Aba, Abia State</t>
   </si>
   <si>
-    <t>Due upon receipt</t>
-  </si>
-  <si>
-    <t>+234 804 678 4565</t>
-  </si>
-  <si>
-    <t>ijegho@ictsl.com</t>
+    <t>COMPANY ACCOUNT DETAILS</t>
+  </si>
+  <si>
+    <t>ICT SOLUTIONS LIMITED</t>
+  </si>
+  <si>
+    <t>Arondizuogu Community Bank =&gt; 20337886565</t>
   </si>
   <si>
     <t>DESCRIPTION</t>
@@ -103,22 +144,10 @@
     <t>AMOUNT</t>
   </si>
   <si>
-    <t>c</t>
-  </si>
-  <si>
-    <t>Helmets</t>
-  </si>
-  <si>
-    <t>Labor: 5 hours at 1800/hr</t>
-  </si>
-  <si>
-    <t>New client discount</t>
-  </si>
-  <si>
-    <t>Dotted Hand Gloves</t>
-  </si>
-  <si>
-    <t>Safety Boots</t>
+    <t>M365 Subscription</t>
+  </si>
+  <si>
+    <t>Internet Service Subscription</t>
   </si>
   <si>
     <t>Thanks for partnering with us.</t>
@@ -150,7 +179,7 @@
     <numFmt numFmtId="164" formatCode="[$₦-470]#,##0.00;\-[$₦-470]#,##0.00"/>
     <numFmt numFmtId="165" formatCode="[$-409]d\-mmm\-yyyy;@"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="16">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -234,6 +263,29 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF242424"/>
+      <name val="Aptos Narrow"/>
+      <charset val="1"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -255,7 +307,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -343,12 +395,21 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment readingOrder="1"/>
@@ -356,22 +417,13 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" readingOrder="1"/>
-    </xf>
     <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment readingOrder="1"/>
     </xf>
     <xf numFmtId="10" fontId="5" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment readingOrder="1"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment readingOrder="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment readingOrder="1"/>
     </xf>
     <xf numFmtId="164" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
@@ -422,16 +474,24 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment readingOrder="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment readingOrder="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="3" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment readingOrder="1"/>
     </xf>
@@ -449,6 +509,9 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" readingOrder="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -466,6 +529,11 @@
           <bgColor rgb="FFF5F5F5"/>
         </patternFill>
       </fill>
+      <border>
+        <right style="thin">
+          <color rgb="FF000000"/>
+        </right>
+      </border>
     </dxf>
     <dxf>
       <font>
@@ -529,7 +597,7 @@
         <shadow val="0"/>
         <u val="none"/>
         <vertAlign val="baseline"/>
-        <sz val="10"/>
+        <sz val="11"/>
         <color theme="1"/>
         <name val="Arial"/>
         <charset val="1"/>
@@ -794,9 +862,15 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <person displayName="Leonard Mbibi" id="{32788DE4-B660-4693-AC8A-21FDCCBD6781}" userId="S::leonard.mbibi@gregobyte.com::02c0729d-909c-4f02-970f-b0082d86fea3" providerId="AD"/>
+</personList>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{CB748B29-1419-4A8B-82C8-2906DFB1F144}" name="InvoiceTable" displayName="InvoiceTable" ref="A15:E21" totalsRowShown="0" headerRowDxfId="14" headerRowBorderDxfId="12" tableBorderDxfId="13" totalsRowBorderDxfId="11">
-  <autoFilter ref="A15:E21" xr:uid="{CB748B29-1419-4A8B-82C8-2906DFB1F144}">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{CB748B29-1419-4A8B-82C8-2906DFB1F144}" name="InvoiceTable" displayName="InvoiceTable" ref="A14:E20" totalsRowShown="0" headerRowDxfId="14" headerRowBorderDxfId="12" tableBorderDxfId="13" totalsRowBorderDxfId="11">
+  <autoFilter ref="A14:E20" xr:uid="{CB748B29-1419-4A8B-82C8-2906DFB1F144}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
@@ -810,22 +884,27 @@
     <tableColumn id="5" xr3:uid="{5E1B32BD-13E3-4DFA-AF31-2B1EA87F074E}" name="AMOUNT" dataDxfId="9">
       <calculatedColumnFormula>IF(OR(InvoiceTable[[#This Row],[UNIT PRICE]]="", InvoiceTable[[#This Row],[DESCRIPTION]]=""), "", IF(InvoiceTable[[#This Row],[QTY]]="", InvoiceTable[[#This Row],[UNIT PRICE]], InvoiceTable[[#This Row],[QTY]]*InvoiceTable[[#This Row],[UNIT PRICE]]))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{C3592BDE-6C53-451A-9DDD-C87FF4C5589F}" name="c" dataDxfId="8"/>
+    <tableColumn id="2" xr3:uid="{C3592BDE-6C53-451A-9DDD-C87FF4C5589F}" name="Row_ID" dataDxfId="8">
+      <calculatedColumnFormula>ROW() - ROW(InvoiceTable[[#Headers],[Row_ID]])</calculatedColumnFormula>
+    </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{EEC8D22E-B88A-42FA-BCA6-0ADB538DF19F}" name="InvoiceNumberTable" displayName="InvoiceNumberTable" ref="A7:E8" totalsRowShown="0" headerRowBorderDxfId="6" tableBorderDxfId="7" totalsRowBorderDxfId="5">
-  <autoFilter ref="A7:E8" xr:uid="{EEC8D22E-B88A-42FA-BCA6-0ADB538DF19F}">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{EEC8D22E-B88A-42FA-BCA6-0ADB538DF19F}" name="InvoiceNumberTable" displayName="InvoiceNumberTable" ref="A7:H8" totalsRowShown="0" headerRowBorderDxfId="6" tableBorderDxfId="7" totalsRowBorderDxfId="5">
+  <autoFilter ref="A7:H8" xr:uid="{EEC8D22E-B88A-42FA-BCA6-0ADB538DF19F}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
     <filterColumn colId="3" hiddenButton="1"/>
     <filterColumn colId="4" hiddenButton="1"/>
+    <filterColumn colId="5" hiddenButton="1"/>
+    <filterColumn colId="6" hiddenButton="1"/>
+    <filterColumn colId="7" hiddenButton="1"/>
   </autoFilter>
-  <tableColumns count="5">
+  <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{44E30872-04A8-4BF4-9D71-76FEC2FAAB2E}" name="BILL_T0" dataDxfId="4"/>
     <tableColumn id="2" xr3:uid="{4977195D-75B6-4433-A4A8-1F9A9F32B3D2}" name="Bill_No" dataDxfId="3"/>
     <tableColumn id="3" xr3:uid="{7845B608-7FC8-4FE3-BB5D-9E412DBBF56B}" name="INVOICE_No" dataDxfId="2"/>
@@ -833,6 +912,9 @@
       <calculatedColumnFormula>TODAY()</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="5" xr3:uid="{F847AC23-4D8D-4B7A-AE33-5F496312EAA1}" name="Row_ID" dataDxfId="0"/>
+    <tableColumn id="6" xr3:uid="{27F3F0F8-987B-4B04-B7E7-6263087FC14B}" name="AddressLine1"/>
+    <tableColumn id="7" xr3:uid="{5579A75A-422C-449B-8425-61A1BAA57925}" name="AddressLine2"/>
+    <tableColumn id="8" xr3:uid="{2AAC3AFA-7A23-4B60-9DF2-DCF9ADF5A78F}" name="AddressLine3"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
 </table>
@@ -1133,63 +1215,73 @@
 </a:theme>
 </file>
 
+<file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
+<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="D21" dT="2026-08-12T14:00:18.67" personId="{32788DE4-B660-4693-AC8A-21FDCCBD6781}" id="{74B194F1-706C-4D16-B8CF-841F3FE0ACD5}">
+    <text>This formula can also be used here:
+=IF(SUM(InvoiceTable[AMOUNT])=0, "", SUM(InvoiceTable[AMOUNT]))</text>
+  </threadedComment>
+</ThreadedComments>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A2:E30"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A2:H29"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="31.42578125" customWidth="1"/>
-    <col min="2" max="2" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="28.28515625" customWidth="1"/>
+    <col min="2" max="2" width="9" customWidth="1"/>
     <col min="3" max="3" width="14.140625" customWidth="1"/>
-    <col min="4" max="4" width="23.42578125" customWidth="1"/>
+    <col min="4" max="4" width="27" customWidth="1"/>
     <col min="5" max="5" width="7.140625" customWidth="1"/>
+    <col min="6" max="8" width="0" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:5" ht="48" customHeight="1">
-      <c r="A2" s="27"/>
-      <c r="B2" s="12"/>
-      <c r="C2" s="36" t="s">
+    <row r="2" spans="1:8" ht="48" customHeight="1">
+      <c r="A2" s="24"/>
+      <c r="B2" s="9"/>
+      <c r="C2" s="37" t="s">
         <v>0</v>
       </c>
-      <c r="D2" s="36"/>
-      <c r="E2" s="24"/>
-    </row>
-    <row r="3" spans="1:5">
-      <c r="A3" s="13" t="s">
+      <c r="D2" s="37"/>
+      <c r="E2" s="21"/>
+    </row>
+    <row r="3" spans="1:8">
+      <c r="A3" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="35"/>
-      <c r="C3" s="35"/>
+      <c r="B3" s="36"/>
+      <c r="C3" s="36"/>
       <c r="D3" s="1"/>
-      <c r="E3" s="21"/>
-    </row>
-    <row r="4" spans="1:5">
-      <c r="A4" s="13" t="s">
+      <c r="E3" s="18"/>
+    </row>
+    <row r="4" spans="1:8">
+      <c r="A4" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="35"/>
-      <c r="C4" s="35"/>
+      <c r="B4" s="36"/>
+      <c r="C4" s="36"/>
       <c r="D4" s="1"/>
-      <c r="E4" s="21"/>
-    </row>
-    <row r="5" spans="1:5">
-      <c r="A5" s="13" t="s">
+      <c r="E4" s="18"/>
+    </row>
+    <row r="5" spans="1:8">
+      <c r="A5" s="10" t="s">
         <v>3</v>
       </c>
       <c r="B5" s="1"/>
       <c r="C5" s="1"/>
       <c r="D5" s="1"/>
-      <c r="E5" s="21"/>
-    </row>
-    <row r="6" spans="1:5">
-      <c r="A6" s="14"/>
+      <c r="E5" s="18"/>
+    </row>
+    <row r="6" spans="1:8">
+      <c r="A6" s="11"/>
       <c r="B6" s="1"/>
       <c r="C6" s="1"/>
-      <c r="D6" s="1"/>
-      <c r="E6" s="21"/>
-    </row>
-    <row r="7" spans="1:5">
-      <c r="A7" s="15" t="s">
+      <c r="D6" s="29"/>
+      <c r="E6" s="18"/>
+    </row>
+    <row r="7" spans="1:8">
+      <c r="A7" s="12" t="s">
         <v>4</v>
       </c>
       <c r="B7" s="2" t="s">
@@ -1201,302 +1293,301 @@
       <c r="D7" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E7" s="25" t="s">
+      <c r="E7" s="22" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="8" spans="1:5">
-      <c r="A8" s="28" t="s">
+      <c r="F7" s="30" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="29">
-        <v>1030</v>
-      </c>
-      <c r="C8" s="30" t="s">
+      <c r="G7" s="31" t="s">
         <v>10</v>
       </c>
-      <c r="D8" s="31">
+      <c r="H7" s="30" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8">
+      <c r="A8" s="25" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8" s="28">
+        <v>1050</v>
+      </c>
+      <c r="C8" s="26" t="s">
+        <v>13</v>
+      </c>
+      <c r="D8" s="27">
         <f ca="1">TODAY()</f>
-        <v>46241</v>
-      </c>
-      <c r="E8" s="32">
+        <v>46249</v>
+      </c>
+      <c r="E8" s="33">
         <v>1</v>
       </c>
-    </row>
-    <row r="9" spans="1:5">
-      <c r="A9" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="B9" s="35"/>
-      <c r="C9" s="35"/>
+      <c r="F8" t="s">
+        <v>14</v>
+      </c>
+      <c r="G8" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8">
+      <c r="A9" s="13" t="str" cm="1">
+        <f t="array" ref="A9">IF(InvoiceNumberTable[AddressLine1] = "", "", InvoiceNumberTable[AddressLine1])</f>
+        <v>12 Ugbana Lane</v>
+      </c>
+      <c r="B9" s="36"/>
+      <c r="C9" s="36"/>
       <c r="D9" s="1"/>
-      <c r="E9" s="21"/>
-    </row>
-    <row r="10" spans="1:5">
-      <c r="A10" s="16" t="s">
-        <v>12</v>
+      <c r="E9" s="18"/>
+    </row>
+    <row r="10" spans="1:8">
+      <c r="A10" s="13" t="str" cm="1">
+        <f t="array" ref="A10">IF(InvoiceNumberTable[AddressLine2] = "", "", InvoiceNumberTable[AddressLine2])</f>
+        <v>Aba, Abia State</v>
       </c>
       <c r="B10" s="1"/>
-      <c r="C10" s="2" t="s">
-        <v>13</v>
-      </c>
+      <c r="C10" s="2"/>
       <c r="D10" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E10" s="26"/>
-    </row>
-    <row r="11" spans="1:5">
-      <c r="A11" s="16" t="s">
-        <v>15</v>
+        <v>16</v>
+      </c>
+      <c r="E10" s="23"/>
+    </row>
+    <row r="11" spans="1:8">
+      <c r="A11" s="13" t="str" cm="1">
+        <f t="array" ref="A11">IF(InvoiceNumberTable[AddressLine3] = "", "", InvoiceNumberTable[AddressLine3])</f>
+        <v/>
       </c>
       <c r="B11" s="1"/>
-      <c r="C11" s="8">
-        <v>100</v>
-      </c>
-      <c r="D11" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="E11" s="21"/>
-    </row>
-    <row r="12" spans="1:5">
-      <c r="A12" s="16" t="s">
+      <c r="C11" s="40" t="s">
         <v>17</v>
       </c>
-      <c r="B12" s="35"/>
-      <c r="C12" s="35"/>
-      <c r="D12" s="1"/>
-      <c r="E12" s="21"/>
-    </row>
-    <row r="13" spans="1:5">
-      <c r="A13" s="17" t="s">
+      <c r="D11" s="40"/>
+      <c r="E11" s="18"/>
+    </row>
+    <row r="12" spans="1:8">
+      <c r="A12" s="14"/>
+      <c r="B12" s="1"/>
+      <c r="C12" s="40" t="s">
         <v>18</v>
       </c>
-      <c r="B13" s="35"/>
-      <c r="C13" s="35"/>
+      <c r="D12" s="40"/>
+      <c r="E12" s="18"/>
+    </row>
+    <row r="13" spans="1:8">
+      <c r="A13" s="11"/>
+      <c r="B13" s="36"/>
+      <c r="C13" s="36"/>
       <c r="D13" s="1"/>
-      <c r="E13" s="21"/>
-    </row>
-    <row r="14" spans="1:5">
-      <c r="A14" s="14"/>
-      <c r="B14" s="35"/>
-      <c r="C14" s="35"/>
-      <c r="D14" s="1"/>
-      <c r="E14" s="21"/>
-    </row>
-    <row r="15" spans="1:5">
-      <c r="A15" s="15" t="s">
+      <c r="E13" s="18"/>
+    </row>
+    <row r="14" spans="1:8">
+      <c r="A14" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="B14" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="C15" s="2" t="s">
+      <c r="C14" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="D15" s="2" t="s">
+      <c r="D14" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="E15" s="25" t="s">
+      <c r="E14" s="22" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8">
+      <c r="A15" s="13" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="16" spans="1:5">
-      <c r="A16" s="16" t="s">
+      <c r="B15" s="5">
+        <v>2</v>
+      </c>
+      <c r="C15" s="3">
+        <v>1700378</v>
+      </c>
+      <c r="D15" s="3">
+        <f>IF(OR(InvoiceTable[[#This Row],[UNIT PRICE]]="", InvoiceTable[[#This Row],[DESCRIPTION]]=""), "", IF(InvoiceTable[[#This Row],[QTY]]="", InvoiceTable[[#This Row],[UNIT PRICE]], InvoiceTable[[#This Row],[QTY]]*InvoiceTable[[#This Row],[UNIT PRICE]]))</f>
+        <v>3400756</v>
+      </c>
+      <c r="E15" s="20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8">
+      <c r="A16" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="B16" s="7">
-        <v>120</v>
-      </c>
-      <c r="C16" s="4">
-        <v>4500</v>
-      </c>
-      <c r="D16" s="4">
+      <c r="B16" s="5">
+        <v>3</v>
+      </c>
+      <c r="C16" s="3">
+        <v>50000</v>
+      </c>
+      <c r="D16" s="3">
         <f>IF(OR(InvoiceTable[[#This Row],[UNIT PRICE]]="", InvoiceTable[[#This Row],[DESCRIPTION]]=""), "", IF(InvoiceTable[[#This Row],[QTY]]="", InvoiceTable[[#This Row],[UNIT PRICE]], InvoiceTable[[#This Row],[QTY]]*InvoiceTable[[#This Row],[UNIT PRICE]]))</f>
-        <v>540000</v>
-      </c>
-      <c r="E16" s="23"/>
+        <v>150000</v>
+      </c>
+      <c r="E16" s="20">
+        <v>2</v>
+      </c>
     </row>
     <row r="17" spans="1:5">
-      <c r="A17" s="16" t="s">
-        <v>25</v>
-      </c>
-      <c r="B17" s="7">
-        <v>5</v>
-      </c>
-      <c r="C17" s="4">
-        <v>75</v>
-      </c>
-      <c r="D17" s="4">
-        <f>IF(OR(InvoiceTable[[#This Row],[UNIT PRICE]]="", InvoiceTable[[#This Row],[DESCRIPTION]]=""), "", IF(InvoiceTable[[#This Row],[QTY]]="", InvoiceTable[[#This Row],[UNIT PRICE]], InvoiceTable[[#This Row],[QTY]]*InvoiceTable[[#This Row],[UNIT PRICE]]))</f>
-        <v>375</v>
-      </c>
-      <c r="E17" s="23"/>
-    </row>
-    <row r="18" spans="1:5">
-      <c r="A18" s="16" t="s">
-        <v>26</v>
-      </c>
-      <c r="B18" s="1"/>
-      <c r="C18" s="4">
-        <v>-50</v>
-      </c>
-      <c r="D18" s="4">
-        <f>IF(OR(InvoiceTable[[#This Row],[UNIT PRICE]]="", InvoiceTable[[#This Row],[DESCRIPTION]]=""), "", IF(InvoiceTable[[#This Row],[QTY]]="", InvoiceTable[[#This Row],[UNIT PRICE]], InvoiceTable[[#This Row],[QTY]]*InvoiceTable[[#This Row],[UNIT PRICE]]))</f>
-        <v>-50</v>
-      </c>
-      <c r="E18" s="23"/>
-    </row>
-    <row r="19" spans="1:5">
-      <c r="A19" s="14" t="s">
-        <v>27</v>
-      </c>
-      <c r="B19" s="1">
-        <v>3</v>
-      </c>
-      <c r="C19" s="4">
-        <v>10000</v>
-      </c>
-      <c r="D19" s="4">
-        <f>IF(OR(InvoiceTable[[#This Row],[UNIT PRICE]]="", InvoiceTable[[#This Row],[DESCRIPTION]]=""), "", IF(InvoiceTable[[#This Row],[QTY]]="", InvoiceTable[[#This Row],[UNIT PRICE]], InvoiceTable[[#This Row],[QTY]]*InvoiceTable[[#This Row],[UNIT PRICE]]))</f>
-        <v>30000</v>
-      </c>
-      <c r="E19" s="23"/>
-    </row>
-    <row r="20" spans="1:5">
-      <c r="A20" s="14" t="s">
-        <v>28</v>
-      </c>
-      <c r="B20" s="1">
-        <v>150</v>
-      </c>
-      <c r="C20" s="9">
-        <v>12000</v>
-      </c>
-      <c r="D20" s="4">
-        <f>IF(OR(InvoiceTable[[#This Row],[UNIT PRICE]]="", InvoiceTable[[#This Row],[DESCRIPTION]]=""), "", IF(InvoiceTable[[#This Row],[QTY]]="", InvoiceTable[[#This Row],[UNIT PRICE]], InvoiceTable[[#This Row],[QTY]]*InvoiceTable[[#This Row],[UNIT PRICE]]))</f>
-        <v>1800000</v>
-      </c>
-      <c r="E20" s="23"/>
-    </row>
-    <row r="21" spans="1:5">
-      <c r="A21" s="14"/>
-      <c r="B21" s="1"/>
-      <c r="C21" s="9"/>
-      <c r="D21" s="4" t="str">
+      <c r="A17" s="13"/>
+      <c r="B17" s="1"/>
+      <c r="C17" s="3"/>
+      <c r="D17" s="3" t="str">
         <f>IF(OR(InvoiceTable[[#This Row],[UNIT PRICE]]="", InvoiceTable[[#This Row],[DESCRIPTION]]=""), "", IF(InvoiceTable[[#This Row],[QTY]]="", InvoiceTable[[#This Row],[UNIT PRICE]], InvoiceTable[[#This Row],[QTY]]*InvoiceTable[[#This Row],[UNIT PRICE]]))</f>
         <v/>
       </c>
-      <c r="E21" s="23"/>
+      <c r="E17" s="20">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5">
+      <c r="A18" s="11"/>
+      <c r="B18" s="1"/>
+      <c r="C18" s="3"/>
+      <c r="D18" s="3" t="str">
+        <f>IF(OR(InvoiceTable[[#This Row],[UNIT PRICE]]="", InvoiceTable[[#This Row],[DESCRIPTION]]=""), "", IF(InvoiceTable[[#This Row],[QTY]]="", InvoiceTable[[#This Row],[UNIT PRICE]], InvoiceTable[[#This Row],[QTY]]*InvoiceTable[[#This Row],[UNIT PRICE]]))</f>
+        <v/>
+      </c>
+      <c r="E18" s="20">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5">
+      <c r="A19" s="11"/>
+      <c r="B19" s="1"/>
+      <c r="C19" s="6"/>
+      <c r="D19" s="3" t="str">
+        <f>IF(OR(InvoiceTable[[#This Row],[UNIT PRICE]]="", InvoiceTable[[#This Row],[DESCRIPTION]]=""), "", IF(InvoiceTable[[#This Row],[QTY]]="", InvoiceTable[[#This Row],[UNIT PRICE]], InvoiceTable[[#This Row],[QTY]]*InvoiceTable[[#This Row],[UNIT PRICE]]))</f>
+        <v/>
+      </c>
+      <c r="E19" s="20">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5">
+      <c r="A20" s="11"/>
+      <c r="B20" s="1"/>
+      <c r="C20" s="6"/>
+      <c r="D20" s="3" t="str">
+        <f>IF(OR(InvoiceTable[[#This Row],[UNIT PRICE]]="", InvoiceTable[[#This Row],[DESCRIPTION]]=""), "", IF(InvoiceTable[[#This Row],[QTY]]="", InvoiceTable[[#This Row],[UNIT PRICE]], InvoiceTable[[#This Row],[QTY]]*InvoiceTable[[#This Row],[UNIT PRICE]]))</f>
+        <v/>
+      </c>
+      <c r="E20" s="20">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5">
+      <c r="A21" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="B21" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="C21" s="5"/>
+      <c r="D21" s="3">
+        <f>IF(INDEX(InvoiceTable[AMOUNT], 1)="", "", SUM(InvoiceTable[AMOUNT]))</f>
+        <v>3550756</v>
+      </c>
+      <c r="E21" s="18"/>
     </row>
     <row r="22" spans="1:5">
-      <c r="A22" s="18" t="s">
+      <c r="A22" s="11"/>
+      <c r="B22" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C22" s="5"/>
+      <c r="D22" s="4">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="E22" s="18"/>
+    </row>
+    <row r="23" spans="1:5">
+      <c r="A23" s="11"/>
+      <c r="B23" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="C23" s="5"/>
+      <c r="D23" s="3">
+        <f>IF(D21="", "", D21 * D22)</f>
+        <v>248552.92</v>
+      </c>
+      <c r="E23" s="18"/>
+    </row>
+    <row r="24" spans="1:5" ht="24">
+      <c r="A24" s="11"/>
+      <c r="B24" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="B22" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="C22" s="7"/>
-      <c r="D22" s="4">
-        <f>SUM(D16:D21)</f>
-        <v>2370325</v>
-      </c>
-      <c r="E22" s="21"/>
-    </row>
-    <row r="23" spans="1:5">
-      <c r="A23" s="14"/>
-      <c r="B23" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="C23" s="7"/>
-      <c r="D23" s="5">
-        <v>7.0000000000000007E-2</v>
-      </c>
-      <c r="E23" s="21"/>
-    </row>
-    <row r="24" spans="1:5">
-      <c r="A24" s="14"/>
-      <c r="B24" s="7" t="s">
-        <v>32</v>
-      </c>
       <c r="C24" s="7"/>
-      <c r="D24" s="4">
-        <f>D23*D22</f>
-        <v>165922.75000000003</v>
-      </c>
-      <c r="E24" s="21"/>
-    </row>
-    <row r="25" spans="1:5" ht="24">
-      <c r="A25" s="14"/>
-      <c r="B25" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="C25" s="10"/>
-      <c r="D25" s="6">
-        <f>D22+D24</f>
-        <v>2536247.75</v>
-      </c>
-      <c r="E25" s="11"/>
+      <c r="D24" s="32">
+        <f>IF(D21 = "", "", D21+D23)</f>
+        <v>3799308.92</v>
+      </c>
+      <c r="E24" s="8"/>
+    </row>
+    <row r="25" spans="1:5">
+      <c r="A25" s="11"/>
+      <c r="B25" s="1"/>
+      <c r="C25" s="1"/>
+      <c r="D25" s="1"/>
+      <c r="E25" s="18"/>
     </row>
     <row r="26" spans="1:5">
-      <c r="A26" s="14"/>
+      <c r="A26" s="11"/>
       <c r="B26" s="1"/>
       <c r="C26" s="1"/>
       <c r="D26" s="1"/>
-      <c r="E26" s="21"/>
+      <c r="E26" s="18"/>
     </row>
     <row r="27" spans="1:5">
-      <c r="A27" s="14"/>
-      <c r="B27" s="1"/>
-      <c r="C27" s="1"/>
-      <c r="D27" s="1"/>
-      <c r="E27" s="21"/>
+      <c r="A27" s="38" t="s">
+        <v>30</v>
+      </c>
+      <c r="B27" s="39"/>
+      <c r="C27" s="39"/>
+      <c r="D27" s="39"/>
+      <c r="E27" s="18"/>
     </row>
     <row r="28" spans="1:5">
-      <c r="A28" s="37" t="s">
-        <v>34</v>
-      </c>
-      <c r="B28" s="38"/>
-      <c r="C28" s="38"/>
-      <c r="D28" s="38"/>
-      <c r="E28" s="21"/>
+      <c r="A28" s="34" t="s">
+        <v>31</v>
+      </c>
+      <c r="B28" s="35"/>
+      <c r="C28" s="35"/>
+      <c r="D28" s="35"/>
+      <c r="E28" s="18"/>
     </row>
     <row r="29" spans="1:5">
-      <c r="A29" s="33" t="s">
-        <v>35</v>
-      </c>
-      <c r="B29" s="34"/>
-      <c r="C29" s="34"/>
-      <c r="D29" s="34"/>
-      <c r="E29" s="21"/>
-    </row>
-    <row r="30" spans="1:5">
-      <c r="A30" s="19"/>
-      <c r="B30" s="20"/>
-      <c r="C30" s="20"/>
-      <c r="D30" s="20"/>
-      <c r="E30" s="22"/>
+      <c r="A29" s="16"/>
+      <c r="B29" s="17"/>
+      <c r="C29" s="17"/>
+      <c r="D29" s="17"/>
+      <c r="E29" s="19"/>
     </row>
   </sheetData>
   <sheetProtection formatCells="0" insertRows="0" autoFilter="0"/>
   <protectedRanges>
-    <protectedRange sqref="A16:C21" name="UserInput"/>
+    <protectedRange sqref="A15:C20" name="UserInput"/>
   </protectedRanges>
   <mergeCells count="9">
-    <mergeCell ref="A29:D29"/>
+    <mergeCell ref="A28:D28"/>
     <mergeCell ref="B13:C13"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="B12:C12"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="B3:C3"/>
     <mergeCell ref="B4:C4"/>
     <mergeCell ref="B9:C9"/>
-    <mergeCell ref="A28:D28"/>
+    <mergeCell ref="A27:D27"/>
+    <mergeCell ref="C11:D11"/>
+    <mergeCell ref="C12:D12"/>
   </mergeCells>
-  <hyperlinks>
-    <hyperlink ref="A13" r:id="rId1" xr:uid="{4467A923-BBDD-4696-987C-7316B9841A21}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId2"/>
+  <drawing r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
   <tableParts count="2">
     <tablePart r:id="rId3"/>
     <tablePart r:id="rId4"/>

</xml_diff>